<commit_message>
updates index e produtos
</commit_message>
<xml_diff>
--- a/Produtos.xlsx
+++ b/Produtos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NOT-MARCOS\Documents\GitHub\Catalogo-Olympikus_2.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8754B9BD-CDB5-4E3B-80A8-2B4F42986356}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08FFE9F6-6F0A-4990-BF8A-721008F252C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12111" uniqueCount="1547">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12111" uniqueCount="1546">
   <si>
     <t>IMAGEM</t>
   </si>
@@ -4285,9 +4285,6 @@
   </si>
   <si>
     <t>OICR261714_FLPSPT</t>
-  </si>
-  <si>
-    <t>cc</t>
   </si>
   <si>
     <t>FLPSPT</t>
@@ -5243,7 +5240,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>35</v>
       </c>
@@ -5350,7 +5347,7 @@
         <v>265.43</v>
       </c>
     </row>
-    <row r="3" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>45</v>
       </c>
@@ -5457,7 +5454,7 @@
         <v>265.43</v>
       </c>
     </row>
-    <row r="4" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>48</v>
       </c>
@@ -5564,7 +5561,7 @@
         <v>265.43</v>
       </c>
     </row>
-    <row r="5" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>50</v>
       </c>
@@ -5671,7 +5668,7 @@
         <v>265.43</v>
       </c>
     </row>
-    <row r="6" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>52</v>
       </c>
@@ -9002,7 +8999,7 @@
         <v>43210417</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>1545</v>
+        <v>1544</v>
       </c>
       <c r="F37" s="4" t="s">
         <v>46</v>
@@ -9109,7 +9106,7 @@
         <v>43210417</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>1545</v>
+        <v>1544</v>
       </c>
       <c r="F38" s="2" t="s">
         <v>46</v>
@@ -9216,7 +9213,7 @@
         <v>43210417</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>1546</v>
+        <v>1545</v>
       </c>
       <c r="F39" s="4" t="s">
         <v>39</v>
@@ -9323,7 +9320,7 @@
         <v>43210417</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>1545</v>
+        <v>1544</v>
       </c>
       <c r="F40" s="2" t="s">
         <v>46</v>
@@ -59250,7 +59247,7 @@
       <c r="AH566" s="4"/>
       <c r="AI566" s="4"/>
     </row>
-    <row r="567" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="567" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A567" s="2" t="s">
         <v>797</v>
       </c>
@@ -59311,7 +59308,7 @@
       <c r="AH567" s="4"/>
       <c r="AI567" s="4"/>
     </row>
-    <row r="568" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="568" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A568" s="2" t="s">
         <v>803</v>
       </c>
@@ -59372,7 +59369,7 @@
       <c r="AH568" s="4"/>
       <c r="AI568" s="4"/>
     </row>
-    <row r="569" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="569" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A569" s="2" t="s">
         <v>804</v>
       </c>
@@ -59433,7 +59430,7 @@
       <c r="AH569" s="4"/>
       <c r="AI569" s="4"/>
     </row>
-    <row r="570" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="570" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A570" s="2" t="s">
         <v>806</v>
       </c>
@@ -59494,7 +59491,7 @@
       <c r="AH570" s="4"/>
       <c r="AI570" s="4"/>
     </row>
-    <row r="571" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="571" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A571" s="2" t="s">
         <v>808</v>
       </c>
@@ -59555,7 +59552,7 @@
       <c r="AH571" s="4"/>
       <c r="AI571" s="4"/>
     </row>
-    <row r="572" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="572" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A572" s="2" t="s">
         <v>810</v>
       </c>
@@ -59616,7 +59613,7 @@
       <c r="AH572" s="4"/>
       <c r="AI572" s="4"/>
     </row>
-    <row r="573" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="573" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A573" s="2" t="s">
         <v>813</v>
       </c>
@@ -59677,7 +59674,7 @@
       <c r="AH573" s="4"/>
       <c r="AI573" s="4"/>
     </row>
-    <row r="574" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="574" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A574" s="2" t="s">
         <v>814</v>
       </c>
@@ -59738,7 +59735,7 @@
       <c r="AH574" s="4"/>
       <c r="AI574" s="4"/>
     </row>
-    <row r="575" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="575" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A575" s="2" t="s">
         <v>815</v>
       </c>
@@ -59799,7 +59796,7 @@
       <c r="AH575" s="4"/>
       <c r="AI575" s="4"/>
     </row>
-    <row r="576" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="576" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A576" s="2" t="s">
         <v>818</v>
       </c>
@@ -59860,7 +59857,7 @@
       <c r="AH576" s="4"/>
       <c r="AI576" s="4"/>
     </row>
-    <row r="577" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="577" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A577" s="2" t="s">
         <v>819</v>
       </c>
@@ -59921,7 +59918,7 @@
       <c r="AH577" s="4"/>
       <c r="AI577" s="4"/>
     </row>
-    <row r="578" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="578" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A578" s="2" t="s">
         <v>820</v>
       </c>
@@ -59982,7 +59979,7 @@
       <c r="AH578" s="4"/>
       <c r="AI578" s="4"/>
     </row>
-    <row r="579" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="579" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A579" s="2" t="s">
         <v>823</v>
       </c>
@@ -60043,7 +60040,7 @@
       <c r="AH579" s="4"/>
       <c r="AI579" s="4"/>
     </row>
-    <row r="580" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="580" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A580" s="2" t="s">
         <v>824</v>
       </c>
@@ -60104,7 +60101,7 @@
       <c r="AH580" s="4"/>
       <c r="AI580" s="4"/>
     </row>
-    <row r="581" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="581" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A581" s="2" t="s">
         <v>825</v>
       </c>
@@ -60165,7 +60162,7 @@
       <c r="AH581" s="4"/>
       <c r="AI581" s="4"/>
     </row>
-    <row r="582" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="582" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A582" s="2" t="s">
         <v>828</v>
       </c>
@@ -60226,7 +60223,7 @@
       <c r="AH582" s="4"/>
       <c r="AI582" s="4"/>
     </row>
-    <row r="583" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="583" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A583" s="2" t="s">
         <v>829</v>
       </c>
@@ -60287,7 +60284,7 @@
       <c r="AH583" s="4"/>
       <c r="AI583" s="4"/>
     </row>
-    <row r="584" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="584" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A584" s="2" t="s">
         <v>830</v>
       </c>
@@ -60348,7 +60345,7 @@
       <c r="AH584" s="4"/>
       <c r="AI584" s="4"/>
     </row>
-    <row r="585" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="585" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A585" s="2" t="s">
         <v>834</v>
       </c>
@@ -60409,7 +60406,7 @@
       <c r="AH585" s="4"/>
       <c r="AI585" s="4"/>
     </row>
-    <row r="586" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="586" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A586" s="2" t="s">
         <v>835</v>
       </c>
@@ -60470,7 +60467,7 @@
       <c r="AH586" s="4"/>
       <c r="AI586" s="4"/>
     </row>
-    <row r="587" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="587" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A587" s="2" t="s">
         <v>836</v>
       </c>
@@ -60531,7 +60528,7 @@
       <c r="AH587" s="4"/>
       <c r="AI587" s="4"/>
     </row>
-    <row r="588" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="588" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A588" s="2" t="s">
         <v>839</v>
       </c>
@@ -60592,7 +60589,7 @@
       <c r="AH588" s="4"/>
       <c r="AI588" s="4"/>
     </row>
-    <row r="589" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="589" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A589" s="2" t="s">
         <v>840</v>
       </c>
@@ -60653,7 +60650,7 @@
       <c r="AH589" s="4"/>
       <c r="AI589" s="4"/>
     </row>
-    <row r="590" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="590" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A590" s="2" t="s">
         <v>841</v>
       </c>
@@ -60714,7 +60711,7 @@
       <c r="AH590" s="4"/>
       <c r="AI590" s="4"/>
     </row>
-    <row r="591" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="591" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A591" s="2" t="s">
         <v>844</v>
       </c>
@@ -60775,7 +60772,7 @@
       <c r="AH591" s="4"/>
       <c r="AI591" s="4"/>
     </row>
-    <row r="592" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="592" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A592" s="2" t="s">
         <v>845</v>
       </c>
@@ -60836,7 +60833,7 @@
       <c r="AH592" s="4"/>
       <c r="AI592" s="4"/>
     </row>
-    <row r="593" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="593" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A593" s="2" t="s">
         <v>846</v>
       </c>
@@ -60897,7 +60894,7 @@
       <c r="AH593" s="4"/>
       <c r="AI593" s="4"/>
     </row>
-    <row r="594" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="594" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A594" s="2" t="s">
         <v>849</v>
       </c>
@@ -60958,7 +60955,7 @@
       <c r="AH594" s="4"/>
       <c r="AI594" s="4"/>
     </row>
-    <row r="595" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="595" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A595" s="2" t="s">
         <v>850</v>
       </c>
@@ -61019,7 +61016,7 @@
       <c r="AH595" s="4"/>
       <c r="AI595" s="4"/>
     </row>
-    <row r="596" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="596" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A596" s="2" t="s">
         <v>851</v>
       </c>
@@ -61080,7 +61077,7 @@
       <c r="AH596" s="4"/>
       <c r="AI596" s="4"/>
     </row>
-    <row r="597" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="597" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A597" s="2" t="s">
         <v>852</v>
       </c>
@@ -61141,7 +61138,7 @@
       <c r="AH597" s="4"/>
       <c r="AI597" s="4"/>
     </row>
-    <row r="598" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="598" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A598" s="2" t="s">
         <v>856</v>
       </c>
@@ -61202,7 +61199,7 @@
       <c r="AH598" s="4"/>
       <c r="AI598" s="4"/>
     </row>
-    <row r="599" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="599" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A599" s="2" t="s">
         <v>857</v>
       </c>
@@ -61263,7 +61260,7 @@
       <c r="AH599" s="4"/>
       <c r="AI599" s="4"/>
     </row>
-    <row r="600" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="600" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A600" s="2" t="s">
         <v>858</v>
       </c>
@@ -61324,7 +61321,7 @@
       <c r="AH600" s="4"/>
       <c r="AI600" s="4"/>
     </row>
-    <row r="601" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="601" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A601" s="2" t="s">
         <v>859</v>
       </c>
@@ -61385,7 +61382,7 @@
       <c r="AH601" s="4"/>
       <c r="AI601" s="4"/>
     </row>
-    <row r="602" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="602" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A602" s="2" t="s">
         <v>860</v>
       </c>
@@ -61446,7 +61443,7 @@
       <c r="AH602" s="4"/>
       <c r="AI602" s="4"/>
     </row>
-    <row r="603" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="603" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A603" s="2" t="s">
         <v>863</v>
       </c>
@@ -61507,7 +61504,7 @@
       <c r="AH603" s="4"/>
       <c r="AI603" s="4"/>
     </row>
-    <row r="604" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="604" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A604" s="2" t="s">
         <v>864</v>
       </c>
@@ -61568,7 +61565,7 @@
       <c r="AH604" s="4"/>
       <c r="AI604" s="4"/>
     </row>
-    <row r="605" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="605" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A605" s="2" t="s">
         <v>865</v>
       </c>
@@ -61629,7 +61626,7 @@
       <c r="AH605" s="4"/>
       <c r="AI605" s="4"/>
     </row>
-    <row r="606" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="606" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A606" s="2" t="s">
         <v>868</v>
       </c>
@@ -61690,7 +61687,7 @@
       <c r="AH606" s="4"/>
       <c r="AI606" s="4"/>
     </row>
-    <row r="607" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="607" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A607" s="2" t="s">
         <v>869</v>
       </c>
@@ -61751,7 +61748,7 @@
       <c r="AH607" s="4"/>
       <c r="AI607" s="4"/>
     </row>
-    <row r="608" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="608" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A608" s="2" t="s">
         <v>870</v>
       </c>
@@ -61812,7 +61809,7 @@
       <c r="AH608" s="4"/>
       <c r="AI608" s="4"/>
     </row>
-    <row r="609" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="609" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A609" s="2" t="s">
         <v>873</v>
       </c>
@@ -61873,7 +61870,7 @@
       <c r="AH609" s="4"/>
       <c r="AI609" s="4"/>
     </row>
-    <row r="610" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="610" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A610" s="2" t="s">
         <v>874</v>
       </c>
@@ -61934,7 +61931,7 @@
       <c r="AH610" s="4"/>
       <c r="AI610" s="4"/>
     </row>
-    <row r="611" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="611" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A611" s="2" t="s">
         <v>875</v>
       </c>
@@ -61995,7 +61992,7 @@
       <c r="AH611" s="4"/>
       <c r="AI611" s="4"/>
     </row>
-    <row r="612" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="612" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A612" s="2" t="s">
         <v>878</v>
       </c>
@@ -62056,7 +62053,7 @@
       <c r="AH612" s="4"/>
       <c r="AI612" s="4"/>
     </row>
-    <row r="613" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="613" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A613" s="2" t="s">
         <v>879</v>
       </c>
@@ -62117,7 +62114,7 @@
       <c r="AH613" s="4"/>
       <c r="AI613" s="4"/>
     </row>
-    <row r="614" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="614" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A614" s="2" t="s">
         <v>880</v>
       </c>
@@ -62178,7 +62175,7 @@
       <c r="AH614" s="4"/>
       <c r="AI614" s="4"/>
     </row>
-    <row r="615" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="615" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A615" s="2" t="s">
         <v>883</v>
       </c>
@@ -62239,7 +62236,7 @@
       <c r="AH615" s="4"/>
       <c r="AI615" s="4"/>
     </row>
-    <row r="616" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="616" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A616" s="2" t="s">
         <v>884</v>
       </c>
@@ -62300,7 +62297,7 @@
       <c r="AH616" s="4"/>
       <c r="AI616" s="4"/>
     </row>
-    <row r="617" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="617" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A617" s="2" t="s">
         <v>885</v>
       </c>
@@ -62361,7 +62358,7 @@
       <c r="AH617" s="4"/>
       <c r="AI617" s="4"/>
     </row>
-    <row r="618" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="618" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A618" s="2" t="s">
         <v>888</v>
       </c>
@@ -62422,7 +62419,7 @@
       <c r="AH618" s="4"/>
       <c r="AI618" s="4"/>
     </row>
-    <row r="619" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="619" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A619" s="2" t="s">
         <v>889</v>
       </c>
@@ -62483,7 +62480,7 @@
       <c r="AH619" s="4"/>
       <c r="AI619" s="4"/>
     </row>
-    <row r="620" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="620" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A620" s="2" t="s">
         <v>890</v>
       </c>
@@ -62544,7 +62541,7 @@
       <c r="AH620" s="4"/>
       <c r="AI620" s="4"/>
     </row>
-    <row r="621" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="621" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A621" s="2" t="s">
         <v>893</v>
       </c>
@@ -62605,7 +62602,7 @@
       <c r="AH621" s="4"/>
       <c r="AI621" s="4"/>
     </row>
-    <row r="622" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="622" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A622" s="2" t="s">
         <v>894</v>
       </c>
@@ -62666,7 +62663,7 @@
       <c r="AH622" s="4"/>
       <c r="AI622" s="4"/>
     </row>
-    <row r="623" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="623" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A623" s="2" t="s">
         <v>895</v>
       </c>
@@ -62727,7 +62724,7 @@
       <c r="AH623" s="4"/>
       <c r="AI623" s="4"/>
     </row>
-    <row r="624" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="624" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A624" s="2" t="s">
         <v>898</v>
       </c>
@@ -62788,7 +62785,7 @@
       <c r="AH624" s="4"/>
       <c r="AI624" s="4"/>
     </row>
-    <row r="625" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="625" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A625" s="2" t="s">
         <v>899</v>
       </c>
@@ -62849,7 +62846,7 @@
       <c r="AH625" s="4"/>
       <c r="AI625" s="4"/>
     </row>
-    <row r="626" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="626" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A626" s="2" t="s">
         <v>900</v>
       </c>
@@ -63154,7 +63151,7 @@
       <c r="AH630" s="4"/>
       <c r="AI630" s="4"/>
     </row>
-    <row r="631" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="631" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A631" s="2" t="s">
         <v>910</v>
       </c>
@@ -63215,7 +63212,7 @@
       <c r="AH631" s="4"/>
       <c r="AI631" s="4"/>
     </row>
-    <row r="632" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="632" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A632" s="2" t="s">
         <v>914</v>
       </c>
@@ -63276,7 +63273,7 @@
       <c r="AH632" s="4"/>
       <c r="AI632" s="4"/>
     </row>
-    <row r="633" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="633" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A633" s="2" t="s">
         <v>916</v>
       </c>
@@ -63337,7 +63334,7 @@
       <c r="AH633" s="4"/>
       <c r="AI633" s="4"/>
     </row>
-    <row r="634" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="634" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A634" s="2" t="s">
         <v>918</v>
       </c>
@@ -63398,7 +63395,7 @@
       <c r="AH634" s="4"/>
       <c r="AI634" s="4"/>
     </row>
-    <row r="635" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="635" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A635" s="2" t="s">
         <v>920</v>
       </c>
@@ -63459,7 +63456,7 @@
       <c r="AH635" s="4"/>
       <c r="AI635" s="4"/>
     </row>
-    <row r="636" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="636" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A636" s="2" t="s">
         <v>922</v>
       </c>
@@ -63520,7 +63517,7 @@
       <c r="AH636" s="4"/>
       <c r="AI636" s="4"/>
     </row>
-    <row r="637" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="637" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A637" s="2" t="s">
         <v>925</v>
       </c>
@@ -63581,7 +63578,7 @@
       <c r="AH637" s="4"/>
       <c r="AI637" s="4"/>
     </row>
-    <row r="638" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="638" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A638" s="2" t="s">
         <v>926</v>
       </c>
@@ -63642,7 +63639,7 @@
       <c r="AH638" s="4"/>
       <c r="AI638" s="4"/>
     </row>
-    <row r="639" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="639" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A639" s="2" t="s">
         <v>927</v>
       </c>
@@ -63703,7 +63700,7 @@
       <c r="AH639" s="4"/>
       <c r="AI639" s="4"/>
     </row>
-    <row r="640" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="640" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A640" s="2" t="s">
         <v>928</v>
       </c>
@@ -66753,7 +66750,7 @@
       <c r="AH689" s="4"/>
       <c r="AI689" s="4"/>
     </row>
-    <row r="690" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="690" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A690" s="2" t="s">
         <v>1025</v>
       </c>
@@ -66814,7 +66811,7 @@
       <c r="AH690" s="4"/>
       <c r="AI690" s="4"/>
     </row>
-    <row r="691" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="691" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A691" s="2" t="s">
         <v>1030</v>
       </c>
@@ -66875,7 +66872,7 @@
       <c r="AH691" s="4"/>
       <c r="AI691" s="4"/>
     </row>
-    <row r="692" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="692" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A692" s="2" t="s">
         <v>1032</v>
       </c>
@@ -66936,7 +66933,7 @@
       <c r="AH692" s="4"/>
       <c r="AI692" s="4"/>
     </row>
-    <row r="693" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="693" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A693" s="2" t="s">
         <v>1036</v>
       </c>
@@ -66997,7 +66994,7 @@
       <c r="AH693" s="4"/>
       <c r="AI693" s="4"/>
     </row>
-    <row r="694" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="694" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A694" s="2" t="s">
         <v>1037</v>
       </c>
@@ -67058,7 +67055,7 @@
       <c r="AH694" s="4"/>
       <c r="AI694" s="4"/>
     </row>
-    <row r="695" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="695" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A695" s="2" t="s">
         <v>1039</v>
       </c>
@@ -67119,7 +67116,7 @@
       <c r="AH695" s="4"/>
       <c r="AI695" s="4"/>
     </row>
-    <row r="696" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="696" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A696" s="2" t="s">
         <v>1042</v>
       </c>
@@ -67180,7 +67177,7 @@
       <c r="AH696" s="4"/>
       <c r="AI696" s="4"/>
     </row>
-    <row r="697" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="697" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A697" s="2" t="s">
         <v>1043</v>
       </c>
@@ -67241,7 +67238,7 @@
       <c r="AH697" s="4"/>
       <c r="AI697" s="4"/>
     </row>
-    <row r="698" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="698" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A698" s="2" t="s">
         <v>1044</v>
       </c>
@@ -67302,7 +67299,7 @@
       <c r="AH698" s="4"/>
       <c r="AI698" s="4"/>
     </row>
-    <row r="699" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="699" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A699" s="2" t="s">
         <v>1046</v>
       </c>
@@ -67363,7 +67360,7 @@
       <c r="AH699" s="4"/>
       <c r="AI699" s="4"/>
     </row>
-    <row r="700" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="700" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A700" s="2" t="s">
         <v>1050</v>
       </c>
@@ -67424,7 +67421,7 @@
       <c r="AH700" s="4"/>
       <c r="AI700" s="4"/>
     </row>
-    <row r="701" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="701" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A701" s="2" t="s">
         <v>1052</v>
       </c>
@@ -67485,7 +67482,7 @@
       <c r="AH701" s="4"/>
       <c r="AI701" s="4"/>
     </row>
-    <row r="702" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="702" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A702" s="2" t="s">
         <v>1055</v>
       </c>
@@ -67546,7 +67543,7 @@
       <c r="AH702" s="4"/>
       <c r="AI702" s="4"/>
     </row>
-    <row r="703" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="703" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A703" s="2" t="s">
         <v>1056</v>
       </c>
@@ -67607,7 +67604,7 @@
       <c r="AH703" s="4"/>
       <c r="AI703" s="4"/>
     </row>
-    <row r="704" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="704" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A704" s="2" t="s">
         <v>1059</v>
       </c>
@@ -67668,7 +67665,7 @@
       <c r="AH704" s="4"/>
       <c r="AI704" s="4"/>
     </row>
-    <row r="705" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="705" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A705" s="2" t="s">
         <v>1060</v>
       </c>
@@ -67685,7 +67682,7 @@
         <v>1034</v>
       </c>
       <c r="F705" s="4" t="s">
-        <v>6</v>
+        <v>855</v>
       </c>
       <c r="G705" s="4" t="s">
         <v>1038</v>
@@ -67729,7 +67726,7 @@
       <c r="AH705" s="4"/>
       <c r="AI705" s="4"/>
     </row>
-    <row r="706" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="706" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A706" s="2" t="s">
         <v>1061</v>
       </c>
@@ -67790,7 +67787,7 @@
       <c r="AH706" s="4"/>
       <c r="AI706" s="4"/>
     </row>
-    <row r="707" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="707" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A707" s="2" t="s">
         <v>1063</v>
       </c>
@@ -67851,7 +67848,7 @@
       <c r="AH707" s="4"/>
       <c r="AI707" s="4"/>
     </row>
-    <row r="708" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="708" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A708" s="2" t="s">
         <v>1064</v>
       </c>
@@ -67912,7 +67909,7 @@
       <c r="AH708" s="4"/>
       <c r="AI708" s="4"/>
     </row>
-    <row r="709" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="709" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A709" s="2" t="s">
         <v>1065</v>
       </c>
@@ -67973,7 +67970,7 @@
       <c r="AH709" s="4"/>
       <c r="AI709" s="4"/>
     </row>
-    <row r="710" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="710" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A710" s="2" t="s">
         <v>1069</v>
       </c>
@@ -68034,7 +68031,7 @@
       <c r="AH710" s="4"/>
       <c r="AI710" s="4"/>
     </row>
-    <row r="711" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="711" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A711" s="2" t="s">
         <v>1071</v>
       </c>
@@ -68095,7 +68092,7 @@
       <c r="AH711" s="4"/>
       <c r="AI711" s="4"/>
     </row>
-    <row r="712" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="712" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A712" s="2" t="s">
         <v>1073</v>
       </c>
@@ -79197,7 +79194,7 @@
       <c r="AH893" s="4"/>
       <c r="AI893" s="4"/>
     </row>
-    <row r="894" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="894" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A894" s="2" t="s">
         <v>1394</v>
       </c>
@@ -79258,7 +79255,7 @@
       <c r="AH894" s="4"/>
       <c r="AI894" s="4"/>
     </row>
-    <row r="895" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="895" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A895" s="2" t="s">
         <v>1397</v>
       </c>
@@ -79319,7 +79316,7 @@
       <c r="AH895" s="4"/>
       <c r="AI895" s="4"/>
     </row>
-    <row r="896" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="896" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A896" s="2" t="s">
         <v>1399</v>
       </c>
@@ -79380,7 +79377,7 @@
       <c r="AH896" s="4"/>
       <c r="AI896" s="4"/>
     </row>
-    <row r="897" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="897" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A897" s="2" t="s">
         <v>1402</v>
       </c>
@@ -79441,7 +79438,7 @@
       <c r="AH897" s="4"/>
       <c r="AI897" s="4"/>
     </row>
-    <row r="898" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="898" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A898" s="2" t="s">
         <v>1404</v>
       </c>
@@ -79502,7 +79499,7 @@
       <c r="AH898" s="4"/>
       <c r="AI898" s="4"/>
     </row>
-    <row r="899" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="899" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A899" s="2" t="s">
         <v>1406</v>
       </c>
@@ -79563,7 +79560,7 @@
       <c r="AH899" s="4"/>
       <c r="AI899" s="4"/>
     </row>
-    <row r="900" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="900" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A900" s="2" t="s">
         <v>1407</v>
       </c>
@@ -79624,7 +79621,7 @@
       <c r="AH900" s="4"/>
       <c r="AI900" s="4"/>
     </row>
-    <row r="901" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="901" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A901" s="2" t="s">
         <v>1410</v>
       </c>
@@ -79751,7 +79748,7 @@
         <v>1415</v>
       </c>
       <c r="B903" s="2" t="s">
-        <v>1416</v>
+        <v>731</v>
       </c>
       <c r="C903" s="2" t="s">
         <v>37</v>
@@ -79766,7 +79763,7 @@
         <v>734</v>
       </c>
       <c r="G903" s="4" t="s">
-        <v>1417</v>
+        <v>1416</v>
       </c>
       <c r="H903" s="4" t="s">
         <v>47</v>
@@ -79807,9 +79804,9 @@
       <c r="AH903" s="4"/>
       <c r="AI903" s="4"/>
     </row>
-    <row r="904" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="904" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A904" s="2" t="s">
-        <v>1418</v>
+        <v>1417</v>
       </c>
       <c r="B904" s="2" t="s">
         <v>798</v>
@@ -79818,16 +79815,16 @@
         <v>37</v>
       </c>
       <c r="D904" s="4" t="s">
+        <v>1418</v>
+      </c>
+      <c r="E904" s="5" t="s">
         <v>1419</v>
-      </c>
-      <c r="E904" s="5" t="s">
-        <v>1420</v>
       </c>
       <c r="F904" s="4" t="s">
         <v>144</v>
       </c>
       <c r="G904" s="4" t="s">
-        <v>1421</v>
+        <v>1420</v>
       </c>
       <c r="H904" s="4" t="s">
         <v>47</v>
@@ -79868,9 +79865,9 @@
       <c r="AH904" s="4"/>
       <c r="AI904" s="4"/>
     </row>
-    <row r="905" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="905" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A905" s="2" t="s">
-        <v>1422</v>
+        <v>1421</v>
       </c>
       <c r="B905" s="2" t="s">
         <v>798</v>
@@ -79879,16 +79876,16 @@
         <v>37</v>
       </c>
       <c r="D905" s="4" t="s">
+        <v>1418</v>
+      </c>
+      <c r="E905" s="5" t="s">
         <v>1419</v>
-      </c>
-      <c r="E905" s="5" t="s">
-        <v>1420</v>
       </c>
       <c r="F905" s="4" t="s">
         <v>144</v>
       </c>
       <c r="G905" s="4" t="s">
-        <v>1423</v>
+        <v>1422</v>
       </c>
       <c r="H905" s="4" t="s">
         <v>47</v>
@@ -79929,9 +79926,9 @@
       <c r="AH905" s="4"/>
       <c r="AI905" s="4"/>
     </row>
-    <row r="906" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="906" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A906" s="2" t="s">
-        <v>1424</v>
+        <v>1423</v>
       </c>
       <c r="B906" s="2" t="s">
         <v>798</v>
@@ -79940,16 +79937,16 @@
         <v>37</v>
       </c>
       <c r="D906" s="4" t="s">
+        <v>1418</v>
+      </c>
+      <c r="E906" s="5" t="s">
         <v>1419</v>
-      </c>
-      <c r="E906" s="5" t="s">
-        <v>1420</v>
       </c>
       <c r="F906" s="4" t="s">
         <v>144</v>
       </c>
       <c r="G906" s="4" t="s">
-        <v>1425</v>
+        <v>1424</v>
       </c>
       <c r="H906" s="4" t="s">
         <v>47</v>
@@ -79990,9 +79987,9 @@
       <c r="AH906" s="4"/>
       <c r="AI906" s="4"/>
     </row>
-    <row r="907" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="907" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A907" s="2" t="s">
-        <v>1426</v>
+        <v>1425</v>
       </c>
       <c r="B907" s="2" t="s">
         <v>798</v>
@@ -80001,16 +79998,16 @@
         <v>37</v>
       </c>
       <c r="D907" s="4" t="s">
+        <v>1426</v>
+      </c>
+      <c r="E907" s="5" t="s">
         <v>1427</v>
-      </c>
-      <c r="E907" s="5" t="s">
-        <v>1428</v>
       </c>
       <c r="F907" s="4" t="s">
         <v>801</v>
       </c>
       <c r="G907" s="4" t="s">
-        <v>1429</v>
+        <v>1428</v>
       </c>
       <c r="H907" s="4" t="s">
         <v>41</v>
@@ -80051,9 +80048,9 @@
       <c r="AH907" s="4"/>
       <c r="AI907" s="4"/>
     </row>
-    <row r="908" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="908" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A908" s="2" t="s">
-        <v>1430</v>
+        <v>1429</v>
       </c>
       <c r="B908" s="2" t="s">
         <v>798</v>
@@ -80062,16 +80059,16 @@
         <v>37</v>
       </c>
       <c r="D908" s="4" t="s">
+        <v>1426</v>
+      </c>
+      <c r="E908" s="5" t="s">
         <v>1427</v>
-      </c>
-      <c r="E908" s="5" t="s">
-        <v>1428</v>
       </c>
       <c r="F908" s="4" t="s">
         <v>801</v>
       </c>
       <c r="G908" s="4" t="s">
-        <v>1431</v>
+        <v>1430</v>
       </c>
       <c r="H908" s="4" t="s">
         <v>41</v>
@@ -80112,9 +80109,9 @@
       <c r="AH908" s="4"/>
       <c r="AI908" s="4"/>
     </row>
-    <row r="909" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="909" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A909" s="2" t="s">
-        <v>1432</v>
+        <v>1431</v>
       </c>
       <c r="B909" s="2" t="s">
         <v>798</v>
@@ -80123,16 +80120,16 @@
         <v>37</v>
       </c>
       <c r="D909" s="4" t="s">
+        <v>1426</v>
+      </c>
+      <c r="E909" s="5" t="s">
         <v>1427</v>
-      </c>
-      <c r="E909" s="5" t="s">
-        <v>1428</v>
       </c>
       <c r="F909" s="4" t="s">
         <v>801</v>
       </c>
       <c r="G909" s="4" t="s">
-        <v>1433</v>
+        <v>1432</v>
       </c>
       <c r="H909" s="4" t="s">
         <v>41</v>
@@ -80173,9 +80170,9 @@
       <c r="AH909" s="4"/>
       <c r="AI909" s="4"/>
     </row>
-    <row r="910" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="910" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A910" s="2" t="s">
-        <v>1434</v>
+        <v>1433</v>
       </c>
       <c r="B910" s="2" t="s">
         <v>798</v>
@@ -80184,16 +80181,16 @@
         <v>37</v>
       </c>
       <c r="D910" s="4" t="s">
+        <v>1426</v>
+      </c>
+      <c r="E910" s="5" t="s">
         <v>1427</v>
-      </c>
-      <c r="E910" s="5" t="s">
-        <v>1428</v>
       </c>
       <c r="F910" s="4" t="s">
         <v>801</v>
       </c>
       <c r="G910" s="4" t="s">
-        <v>1435</v>
+        <v>1434</v>
       </c>
       <c r="H910" s="4" t="s">
         <v>41</v>
@@ -80234,9 +80231,9 @@
       <c r="AH910" s="4"/>
       <c r="AI910" s="4"/>
     </row>
-    <row r="911" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="911" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A911" s="2" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="B911" s="2" t="s">
         <v>798</v>
@@ -80245,16 +80242,16 @@
         <v>37</v>
       </c>
       <c r="D911" s="4" t="s">
+        <v>1436</v>
+      </c>
+      <c r="E911" s="5" t="s">
         <v>1437</v>
-      </c>
-      <c r="E911" s="5" t="s">
-        <v>1438</v>
       </c>
       <c r="F911" s="4" t="s">
         <v>855</v>
       </c>
       <c r="G911" s="4" t="s">
-        <v>1429</v>
+        <v>1428</v>
       </c>
       <c r="H911" s="4" t="s">
         <v>96</v>
@@ -80295,9 +80292,9 @@
       <c r="AH911" s="4"/>
       <c r="AI911" s="4"/>
     </row>
-    <row r="912" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="912" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A912" s="2" t="s">
-        <v>1439</v>
+        <v>1438</v>
       </c>
       <c r="B912" s="2" t="s">
         <v>798</v>
@@ -80306,16 +80303,16 @@
         <v>37</v>
       </c>
       <c r="D912" s="4" t="s">
+        <v>1436</v>
+      </c>
+      <c r="E912" s="5" t="s">
         <v>1437</v>
-      </c>
-      <c r="E912" s="5" t="s">
-        <v>1438</v>
       </c>
       <c r="F912" s="4" t="s">
         <v>855</v>
       </c>
       <c r="G912" s="4" t="s">
-        <v>1431</v>
+        <v>1430</v>
       </c>
       <c r="H912" s="4" t="s">
         <v>96</v>
@@ -80356,9 +80353,9 @@
       <c r="AH912" s="4"/>
       <c r="AI912" s="4"/>
     </row>
-    <row r="913" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="913" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A913" s="2" t="s">
-        <v>1440</v>
+        <v>1439</v>
       </c>
       <c r="B913" s="2" t="s">
         <v>798</v>
@@ -80367,16 +80364,16 @@
         <v>37</v>
       </c>
       <c r="D913" s="4" t="s">
+        <v>1436</v>
+      </c>
+      <c r="E913" s="5" t="s">
         <v>1437</v>
-      </c>
-      <c r="E913" s="5" t="s">
-        <v>1438</v>
       </c>
       <c r="F913" s="4" t="s">
         <v>855</v>
       </c>
       <c r="G913" s="4" t="s">
-        <v>1433</v>
+        <v>1432</v>
       </c>
       <c r="H913" s="4" t="s">
         <v>96</v>
@@ -80417,9 +80414,9 @@
       <c r="AH913" s="4"/>
       <c r="AI913" s="4"/>
     </row>
-    <row r="914" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="914" spans="1:35" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A914" s="2" t="s">
-        <v>1441</v>
+        <v>1440</v>
       </c>
       <c r="B914" s="2" t="s">
         <v>798</v>
@@ -80428,16 +80425,16 @@
         <v>37</v>
       </c>
       <c r="D914" s="4" t="s">
+        <v>1436</v>
+      </c>
+      <c r="E914" s="5" t="s">
         <v>1437</v>
-      </c>
-      <c r="E914" s="5" t="s">
-        <v>1438</v>
       </c>
       <c r="F914" s="4" t="s">
         <v>855</v>
       </c>
       <c r="G914" s="4" t="s">
-        <v>1435</v>
+        <v>1434</v>
       </c>
       <c r="H914" s="4" t="s">
         <v>96</v>
@@ -80480,7 +80477,7 @@
     </row>
     <row r="915" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A915" s="2" t="s">
-        <v>1442</v>
+        <v>1441</v>
       </c>
       <c r="B915" s="2" t="s">
         <v>700</v>
@@ -80489,10 +80486,10 @@
         <v>110</v>
       </c>
       <c r="D915" s="4" t="s">
+        <v>1442</v>
+      </c>
+      <c r="E915" s="5" t="s">
         <v>1443</v>
-      </c>
-      <c r="E915" s="5" t="s">
-        <v>1444</v>
       </c>
       <c r="F915" s="4" t="s">
         <v>1364</v>
@@ -80541,7 +80538,7 @@
     </row>
     <row r="916" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A916" s="2" t="s">
-        <v>1445</v>
+        <v>1444</v>
       </c>
       <c r="B916" s="2" t="s">
         <v>700</v>
@@ -80550,10 +80547,10 @@
         <v>110</v>
       </c>
       <c r="D916" s="4" t="s">
+        <v>1442</v>
+      </c>
+      <c r="E916" s="5" t="s">
         <v>1443</v>
-      </c>
-      <c r="E916" s="5" t="s">
-        <v>1444</v>
       </c>
       <c r="F916" s="4" t="s">
         <v>1364</v>
@@ -80602,7 +80599,7 @@
     </row>
     <row r="917" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A917" s="2" t="s">
-        <v>1446</v>
+        <v>1445</v>
       </c>
       <c r="B917" s="2" t="s">
         <v>700</v>
@@ -80611,10 +80608,10 @@
         <v>110</v>
       </c>
       <c r="D917" s="4" t="s">
+        <v>1446</v>
+      </c>
+      <c r="E917" s="5" t="s">
         <v>1447</v>
-      </c>
-      <c r="E917" s="5" t="s">
-        <v>1448</v>
       </c>
       <c r="F917" s="4" t="s">
         <v>1364</v>
@@ -80663,7 +80660,7 @@
     </row>
     <row r="918" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A918" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="B918" s="2" t="s">
         <v>700</v>
@@ -80672,10 +80669,10 @@
         <v>110</v>
       </c>
       <c r="D918" s="4" t="s">
+        <v>1446</v>
+      </c>
+      <c r="E918" s="5" t="s">
         <v>1447</v>
-      </c>
-      <c r="E918" s="5" t="s">
-        <v>1448</v>
       </c>
       <c r="F918" s="4" t="s">
         <v>1364</v>
@@ -80724,7 +80721,7 @@
     </row>
     <row r="919" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A919" s="2" t="s">
-        <v>1450</v>
+        <v>1449</v>
       </c>
       <c r="B919" s="2" t="s">
         <v>700</v>
@@ -80733,10 +80730,10 @@
         <v>110</v>
       </c>
       <c r="D919" s="4" t="s">
+        <v>1450</v>
+      </c>
+      <c r="E919" s="5" t="s">
         <v>1451</v>
-      </c>
-      <c r="E919" s="5" t="s">
-        <v>1452</v>
       </c>
       <c r="F919" s="4" t="s">
         <v>710</v>
@@ -80785,7 +80782,7 @@
     </row>
     <row r="920" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A920" s="2" t="s">
-        <v>1453</v>
+        <v>1452</v>
       </c>
       <c r="B920" s="2" t="s">
         <v>700</v>
@@ -80794,10 +80791,10 @@
         <v>110</v>
       </c>
       <c r="D920" s="4" t="s">
+        <v>1450</v>
+      </c>
+      <c r="E920" s="5" t="s">
         <v>1451</v>
-      </c>
-      <c r="E920" s="5" t="s">
-        <v>1452</v>
       </c>
       <c r="F920" s="4" t="s">
         <v>710</v>
@@ -80846,7 +80843,7 @@
     </row>
     <row r="921" spans="1:35" ht="18.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A921" s="2" t="s">
-        <v>1454</v>
+        <v>1453</v>
       </c>
       <c r="B921" s="2" t="s">
         <v>700</v>
@@ -80855,10 +80852,10 @@
         <v>110</v>
       </c>
       <c r="D921" s="4" t="s">
+        <v>1450</v>
+      </c>
+      <c r="E921" s="5" t="s">
         <v>1451</v>
-      </c>
-      <c r="E921" s="5" t="s">
-        <v>1452</v>
       </c>
       <c r="F921" s="4" t="s">
         <v>710</v>
@@ -80907,9 +80904,9 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:R921" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <filterColumn colId="4">
+    <filterColumn colId="1">
       <filters>
-        <filter val="CARDIO"/>
+        <filter val="MEIA"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -80987,10 +80984,10 @@
         <v>593</v>
       </c>
       <c r="D2" s="4" t="s">
+        <v>1454</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>1455</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>1456</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>710</v>
@@ -81029,10 +81026,10 @@
         <v>593</v>
       </c>
       <c r="D3" s="4" t="s">
+        <v>1456</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>1457</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>1458</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>710</v>
@@ -81071,16 +81068,16 @@
         <v>37</v>
       </c>
       <c r="D4" s="4" t="s">
+        <v>1458</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>1459</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>1460</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>1145</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>1461</v>
+        <v>1460</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>41</v>
@@ -81113,10 +81110,10 @@
         <v>37</v>
       </c>
       <c r="D5" s="4" t="s">
+        <v>1458</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>1459</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>1460</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>1145</v>
@@ -81155,16 +81152,16 @@
         <v>37</v>
       </c>
       <c r="D6" s="4" t="s">
+        <v>1461</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>1462</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>1463</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>1145</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>1464</v>
+        <v>1463</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>41</v>
@@ -81197,16 +81194,16 @@
         <v>37</v>
       </c>
       <c r="D7" s="4" t="s">
+        <v>1461</v>
+      </c>
+      <c r="E7" s="5" t="s">
         <v>1462</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>1463</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>1145</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>1465</v>
+        <v>1464</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>41</v>
@@ -81239,10 +81236,10 @@
         <v>37</v>
       </c>
       <c r="D8" s="4" t="s">
+        <v>1461</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>1462</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>1463</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>1145</v>
@@ -81281,16 +81278,16 @@
         <v>37</v>
       </c>
       <c r="D9" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>1466</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>1467</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>1145</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>1468</v>
+        <v>1467</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>41</v>
@@ -81323,16 +81320,16 @@
         <v>37</v>
       </c>
       <c r="D10" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>1466</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>1467</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>1145</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>1465</v>
+        <v>1464</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>41</v>
@@ -81365,16 +81362,16 @@
         <v>37</v>
       </c>
       <c r="D11" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="E11" s="5" t="s">
         <v>1466</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>1467</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>1145</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>1464</v>
+        <v>1463</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>41</v>
@@ -81407,10 +81404,10 @@
         <v>37</v>
       </c>
       <c r="D12" s="4" t="s">
+        <v>1465</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>1466</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>1467</v>
       </c>
       <c r="F12" s="4" t="s">
         <v>1145</v>
@@ -81449,10 +81446,10 @@
         <v>37</v>
       </c>
       <c r="D13" s="4" t="s">
+        <v>1468</v>
+      </c>
+      <c r="E13" s="5" t="s">
         <v>1469</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>1470</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>1145</v>
@@ -81491,16 +81488,16 @@
         <v>37</v>
       </c>
       <c r="D14" s="4" t="s">
+        <v>1468</v>
+      </c>
+      <c r="E14" s="5" t="s">
         <v>1469</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>1470</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>1145</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>1461</v>
+        <v>1460</v>
       </c>
       <c r="H14" s="4" t="s">
         <v>41</v>
@@ -81533,16 +81530,16 @@
         <v>37</v>
       </c>
       <c r="D15" s="4" t="s">
+        <v>1468</v>
+      </c>
+      <c r="E15" s="5" t="s">
         <v>1469</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>1470</v>
       </c>
       <c r="F15" s="4" t="s">
         <v>1145</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>1465</v>
+        <v>1464</v>
       </c>
       <c r="H15" s="4" t="s">
         <v>41</v>
@@ -81575,16 +81572,16 @@
         <v>37</v>
       </c>
       <c r="D16" s="4" t="s">
+        <v>1470</v>
+      </c>
+      <c r="E16" s="5" t="s">
         <v>1471</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>1472</v>
       </c>
       <c r="F16" s="4" t="s">
         <v>1145</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>1468</v>
+        <v>1467</v>
       </c>
       <c r="H16" s="4" t="s">
         <v>41</v>
@@ -81617,16 +81614,16 @@
         <v>37</v>
       </c>
       <c r="D17" s="4" t="s">
+        <v>1470</v>
+      </c>
+      <c r="E17" s="5" t="s">
         <v>1471</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>1472</v>
       </c>
       <c r="F17" s="4" t="s">
         <v>1145</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>1465</v>
+        <v>1464</v>
       </c>
       <c r="H17" s="4" t="s">
         <v>41</v>
@@ -81659,10 +81656,10 @@
         <v>37</v>
       </c>
       <c r="D18" s="4" t="s">
+        <v>1472</v>
+      </c>
+      <c r="E18" s="5" t="s">
         <v>1473</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>1474</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>1145</v>
@@ -81701,16 +81698,16 @@
         <v>37</v>
       </c>
       <c r="D19" s="4" t="s">
+        <v>1472</v>
+      </c>
+      <c r="E19" s="5" t="s">
         <v>1473</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>1474</v>
       </c>
       <c r="F19" s="4" t="s">
         <v>1145</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>1461</v>
+        <v>1460</v>
       </c>
       <c r="H19" s="4" t="s">
         <v>41</v>
@@ -81743,10 +81740,10 @@
         <v>37</v>
       </c>
       <c r="D20" s="4" t="s">
+        <v>1474</v>
+      </c>
+      <c r="E20" s="5" t="s">
         <v>1475</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>1476</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>1145</v>
@@ -81785,10 +81782,10 @@
         <v>37</v>
       </c>
       <c r="D21" s="4" t="s">
+        <v>1474</v>
+      </c>
+      <c r="E21" s="5" t="s">
         <v>1475</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>1476</v>
       </c>
       <c r="F21" s="4" t="s">
         <v>1145</v>
@@ -81827,10 +81824,10 @@
         <v>37</v>
       </c>
       <c r="D22" s="4" t="s">
+        <v>1476</v>
+      </c>
+      <c r="E22" s="5" t="s">
         <v>1477</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>1478</v>
       </c>
       <c r="F22" s="4" t="s">
         <v>1145</v>
@@ -81869,16 +81866,16 @@
         <v>37</v>
       </c>
       <c r="D23" s="4" t="s">
+        <v>1476</v>
+      </c>
+      <c r="E23" s="5" t="s">
         <v>1477</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>1478</v>
       </c>
       <c r="F23" s="4" t="s">
         <v>1145</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>1468</v>
+        <v>1467</v>
       </c>
       <c r="H23" s="4" t="s">
         <v>96</v>
@@ -81911,16 +81908,16 @@
         <v>37</v>
       </c>
       <c r="D24" s="4" t="s">
+        <v>1476</v>
+      </c>
+      <c r="E24" s="5" t="s">
         <v>1477</v>
-      </c>
-      <c r="E24" s="5" t="s">
-        <v>1478</v>
       </c>
       <c r="F24" s="4" t="s">
         <v>1145</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>1464</v>
+        <v>1463</v>
       </c>
       <c r="H24" s="4" t="s">
         <v>96</v>
@@ -81953,16 +81950,16 @@
         <v>37</v>
       </c>
       <c r="D25" s="4" t="s">
+        <v>1476</v>
+      </c>
+      <c r="E25" s="5" t="s">
         <v>1477</v>
-      </c>
-      <c r="E25" s="5" t="s">
-        <v>1478</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>1145</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>1479</v>
+        <v>1478</v>
       </c>
       <c r="H25" s="4" t="s">
         <v>96</v>
@@ -81995,16 +81992,16 @@
         <v>37</v>
       </c>
       <c r="D26" s="4" t="s">
+        <v>1479</v>
+      </c>
+      <c r="E26" s="5" t="s">
         <v>1480</v>
-      </c>
-      <c r="E26" s="5" t="s">
-        <v>1481</v>
       </c>
       <c r="F26" s="4" t="s">
         <v>1145</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>1461</v>
+        <v>1460</v>
       </c>
       <c r="H26" s="4" t="s">
         <v>96</v>
@@ -82037,16 +82034,16 @@
         <v>37</v>
       </c>
       <c r="D27" s="4" t="s">
+        <v>1479</v>
+      </c>
+      <c r="E27" s="5" t="s">
         <v>1480</v>
-      </c>
-      <c r="E27" s="5" t="s">
-        <v>1481</v>
       </c>
       <c r="F27" s="4" t="s">
         <v>1145</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>1479</v>
+        <v>1478</v>
       </c>
       <c r="H27" s="4" t="s">
         <v>96</v>
@@ -82079,16 +82076,16 @@
         <v>37</v>
       </c>
       <c r="D28" s="4" t="s">
+        <v>1479</v>
+      </c>
+      <c r="E28" s="5" t="s">
         <v>1480</v>
-      </c>
-      <c r="E28" s="5" t="s">
-        <v>1481</v>
       </c>
       <c r="F28" s="4" t="s">
         <v>1145</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>1482</v>
+        <v>1481</v>
       </c>
       <c r="H28" s="4" t="s">
         <v>96</v>
@@ -82121,10 +82118,10 @@
         <v>37</v>
       </c>
       <c r="D29" s="4" t="s">
+        <v>1479</v>
+      </c>
+      <c r="E29" s="5" t="s">
         <v>1480</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>1481</v>
       </c>
       <c r="F29" s="4" t="s">
         <v>1145</v>
@@ -82163,10 +82160,10 @@
         <v>37</v>
       </c>
       <c r="D30" s="4" t="s">
+        <v>1482</v>
+      </c>
+      <c r="E30" s="5" t="s">
         <v>1483</v>
-      </c>
-      <c r="E30" s="5" t="s">
-        <v>1484</v>
       </c>
       <c r="F30" s="4" t="s">
         <v>1145</v>
@@ -82205,10 +82202,10 @@
         <v>37</v>
       </c>
       <c r="D31" s="4" t="s">
+        <v>1482</v>
+      </c>
+      <c r="E31" s="5" t="s">
         <v>1483</v>
-      </c>
-      <c r="E31" s="5" t="s">
-        <v>1484</v>
       </c>
       <c r="F31" s="4" t="s">
         <v>1145</v>
@@ -82247,16 +82244,16 @@
         <v>37</v>
       </c>
       <c r="D32" s="4" t="s">
+        <v>1482</v>
+      </c>
+      <c r="E32" s="5" t="s">
         <v>1483</v>
-      </c>
-      <c r="E32" s="5" t="s">
-        <v>1484</v>
       </c>
       <c r="F32" s="4" t="s">
         <v>1145</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>1461</v>
+        <v>1460</v>
       </c>
       <c r="H32" s="4" t="s">
         <v>96</v>
@@ -82289,10 +82286,10 @@
         <v>37</v>
       </c>
       <c r="D33" s="4" t="s">
+        <v>1484</v>
+      </c>
+      <c r="E33" s="5" t="s">
         <v>1485</v>
-      </c>
-      <c r="E33" s="5" t="s">
-        <v>1486</v>
       </c>
       <c r="F33" s="4" t="s">
         <v>6</v>
@@ -82331,10 +82328,10 @@
         <v>37</v>
       </c>
       <c r="D34" s="4" t="s">
+        <v>1486</v>
+      </c>
+      <c r="E34" s="5" t="s">
         <v>1487</v>
-      </c>
-      <c r="E34" s="5" t="s">
-        <v>1488</v>
       </c>
       <c r="F34" s="4" t="s">
         <v>1145</v>
@@ -82373,10 +82370,10 @@
         <v>37</v>
       </c>
       <c r="D35" s="4" t="s">
+        <v>1486</v>
+      </c>
+      <c r="E35" s="5" t="s">
         <v>1487</v>
-      </c>
-      <c r="E35" s="5" t="s">
-        <v>1488</v>
       </c>
       <c r="F35" s="4" t="s">
         <v>1145</v>
@@ -82415,10 +82412,10 @@
         <v>37</v>
       </c>
       <c r="D36" s="4" t="s">
+        <v>1488</v>
+      </c>
+      <c r="E36" s="5" t="s">
         <v>1489</v>
-      </c>
-      <c r="E36" s="5" t="s">
-        <v>1490</v>
       </c>
       <c r="F36" s="4" t="s">
         <v>734</v>
@@ -82457,10 +82454,10 @@
         <v>37</v>
       </c>
       <c r="D37" s="4" t="s">
+        <v>1488</v>
+      </c>
+      <c r="E37" s="5" t="s">
         <v>1489</v>
-      </c>
-      <c r="E37" s="5" t="s">
-        <v>1490</v>
       </c>
       <c r="F37" s="4" t="s">
         <v>734</v>
@@ -82499,10 +82496,10 @@
         <v>37</v>
       </c>
       <c r="D38" s="4" t="s">
+        <v>1490</v>
+      </c>
+      <c r="E38" s="5" t="s">
         <v>1491</v>
-      </c>
-      <c r="E38" s="5" t="s">
-        <v>1492</v>
       </c>
       <c r="F38" s="4" t="s">
         <v>1145</v>
@@ -82541,10 +82538,10 @@
         <v>37</v>
       </c>
       <c r="D39" s="4" t="s">
+        <v>1490</v>
+      </c>
+      <c r="E39" s="5" t="s">
         <v>1491</v>
-      </c>
-      <c r="E39" s="5" t="s">
-        <v>1492</v>
       </c>
       <c r="F39" s="4" t="s">
         <v>1145</v>
@@ -82583,10 +82580,10 @@
         <v>37</v>
       </c>
       <c r="D40" s="4" t="s">
+        <v>1492</v>
+      </c>
+      <c r="E40" s="5" t="s">
         <v>1493</v>
-      </c>
-      <c r="E40" s="5" t="s">
-        <v>1494</v>
       </c>
       <c r="F40" s="4" t="s">
         <v>1145</v>
@@ -82625,16 +82622,16 @@
         <v>37</v>
       </c>
       <c r="D41" s="4" t="s">
+        <v>1492</v>
+      </c>
+      <c r="E41" s="5" t="s">
         <v>1493</v>
-      </c>
-      <c r="E41" s="5" t="s">
-        <v>1494</v>
       </c>
       <c r="F41" s="4" t="s">
         <v>1145</v>
       </c>
       <c r="G41" s="4" t="s">
-        <v>1495</v>
+        <v>1494</v>
       </c>
       <c r="H41" s="4" t="s">
         <v>41</v>
@@ -82667,10 +82664,10 @@
         <v>37</v>
       </c>
       <c r="D42" s="4" t="s">
+        <v>1495</v>
+      </c>
+      <c r="E42" s="5" t="s">
         <v>1496</v>
-      </c>
-      <c r="E42" s="5" t="s">
-        <v>1497</v>
       </c>
       <c r="F42" s="4" t="s">
         <v>1145</v>
@@ -82709,10 +82706,10 @@
         <v>37</v>
       </c>
       <c r="D43" s="4" t="s">
+        <v>1495</v>
+      </c>
+      <c r="E43" s="5" t="s">
         <v>1496</v>
-      </c>
-      <c r="E43" s="5" t="s">
-        <v>1497</v>
       </c>
       <c r="F43" s="4" t="s">
         <v>1145</v>
@@ -82751,16 +82748,16 @@
         <v>37</v>
       </c>
       <c r="D44" s="4" t="s">
+        <v>1497</v>
+      </c>
+      <c r="E44" s="5" t="s">
         <v>1498</v>
-      </c>
-      <c r="E44" s="5" t="s">
-        <v>1499</v>
       </c>
       <c r="F44" s="4" t="s">
         <v>1145</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>1425</v>
+        <v>1424</v>
       </c>
       <c r="H44" s="4" t="s">
         <v>41</v>
@@ -82793,10 +82790,10 @@
         <v>37</v>
       </c>
       <c r="D45" s="4" t="s">
+        <v>1497</v>
+      </c>
+      <c r="E45" s="5" t="s">
         <v>1498</v>
-      </c>
-      <c r="E45" s="5" t="s">
-        <v>1499</v>
       </c>
       <c r="F45" s="4" t="s">
         <v>1145</v>
@@ -82835,10 +82832,10 @@
         <v>37</v>
       </c>
       <c r="D46" s="4" t="s">
+        <v>1499</v>
+      </c>
+      <c r="E46" s="5" t="s">
         <v>1500</v>
-      </c>
-      <c r="E46" s="5" t="s">
-        <v>1501</v>
       </c>
       <c r="F46" s="4" t="s">
         <v>1145</v>
@@ -82877,16 +82874,16 @@
         <v>37</v>
       </c>
       <c r="D47" s="4" t="s">
+        <v>1499</v>
+      </c>
+      <c r="E47" s="5" t="s">
         <v>1500</v>
-      </c>
-      <c r="E47" s="5" t="s">
-        <v>1501</v>
       </c>
       <c r="F47" s="4" t="s">
         <v>1145</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>1495</v>
+        <v>1494</v>
       </c>
       <c r="H47" s="4" t="s">
         <v>41</v>
@@ -82919,10 +82916,10 @@
         <v>37</v>
       </c>
       <c r="D48" s="4" t="s">
+        <v>1499</v>
+      </c>
+      <c r="E48" s="5" t="s">
         <v>1500</v>
-      </c>
-      <c r="E48" s="5" t="s">
-        <v>1501</v>
       </c>
       <c r="F48" s="4" t="s">
         <v>1145</v>
@@ -82961,10 +82958,10 @@
         <v>37</v>
       </c>
       <c r="D49" s="4" t="s">
+        <v>1501</v>
+      </c>
+      <c r="E49" s="5" t="s">
         <v>1502</v>
-      </c>
-      <c r="E49" s="5" t="s">
-        <v>1503</v>
       </c>
       <c r="F49" s="4" t="s">
         <v>1145</v>
@@ -83003,10 +83000,10 @@
         <v>37</v>
       </c>
       <c r="D50" s="4" t="s">
+        <v>1501</v>
+      </c>
+      <c r="E50" s="5" t="s">
         <v>1502</v>
-      </c>
-      <c r="E50" s="5" t="s">
-        <v>1503</v>
       </c>
       <c r="F50" s="4" t="s">
         <v>1145</v>
@@ -83045,10 +83042,10 @@
         <v>37</v>
       </c>
       <c r="D51" s="4" t="s">
+        <v>1503</v>
+      </c>
+      <c r="E51" s="5" t="s">
         <v>1504</v>
-      </c>
-      <c r="E51" s="5" t="s">
-        <v>1505</v>
       </c>
       <c r="F51" s="4" t="s">
         <v>1145</v>
@@ -83087,16 +83084,16 @@
         <v>37</v>
       </c>
       <c r="D52" s="4" t="s">
+        <v>1503</v>
+      </c>
+      <c r="E52" s="5" t="s">
         <v>1504</v>
-      </c>
-      <c r="E52" s="5" t="s">
-        <v>1505</v>
       </c>
       <c r="F52" s="4" t="s">
         <v>1145</v>
       </c>
       <c r="G52" s="4" t="s">
-        <v>1495</v>
+        <v>1494</v>
       </c>
       <c r="H52" s="4" t="s">
         <v>41</v>
@@ -83129,10 +83126,10 @@
         <v>37</v>
       </c>
       <c r="D53" s="4" t="s">
+        <v>1505</v>
+      </c>
+      <c r="E53" s="5" t="s">
         <v>1506</v>
-      </c>
-      <c r="E53" s="5" t="s">
-        <v>1507</v>
       </c>
       <c r="F53" s="4" t="s">
         <v>1145</v>
@@ -83171,10 +83168,10 @@
         <v>37</v>
       </c>
       <c r="D54" s="4" t="s">
+        <v>1505</v>
+      </c>
+      <c r="E54" s="5" t="s">
         <v>1506</v>
-      </c>
-      <c r="E54" s="5" t="s">
-        <v>1507</v>
       </c>
       <c r="F54" s="4" t="s">
         <v>1145</v>
@@ -83213,10 +83210,10 @@
         <v>37</v>
       </c>
       <c r="D55" s="4" t="s">
+        <v>1507</v>
+      </c>
+      <c r="E55" s="5" t="s">
         <v>1508</v>
-      </c>
-      <c r="E55" s="5" t="s">
-        <v>1509</v>
       </c>
       <c r="F55" s="4" t="s">
         <v>1145</v>
@@ -83255,16 +83252,16 @@
         <v>37</v>
       </c>
       <c r="D56" s="4" t="s">
+        <v>1509</v>
+      </c>
+      <c r="E56" s="5" t="s">
         <v>1510</v>
-      </c>
-      <c r="E56" s="5" t="s">
-        <v>1511</v>
       </c>
       <c r="F56" s="4" t="s">
         <v>1145</v>
       </c>
       <c r="G56" s="4" t="s">
-        <v>1425</v>
+        <v>1424</v>
       </c>
       <c r="H56" s="4" t="s">
         <v>96</v>
@@ -83297,10 +83294,10 @@
         <v>37</v>
       </c>
       <c r="D57" s="4" t="s">
+        <v>1509</v>
+      </c>
+      <c r="E57" s="5" t="s">
         <v>1510</v>
-      </c>
-      <c r="E57" s="5" t="s">
-        <v>1511</v>
       </c>
       <c r="F57" s="4" t="s">
         <v>1145</v>
@@ -83339,10 +83336,10 @@
         <v>37</v>
       </c>
       <c r="D58" s="4" t="s">
+        <v>1511</v>
+      </c>
+      <c r="E58" s="5" t="s">
         <v>1512</v>
-      </c>
-      <c r="E58" s="5" t="s">
-        <v>1513</v>
       </c>
       <c r="F58" s="4" t="s">
         <v>1145</v>
@@ -83381,10 +83378,10 @@
         <v>37</v>
       </c>
       <c r="D59" s="4" t="s">
+        <v>1511</v>
+      </c>
+      <c r="E59" s="5" t="s">
         <v>1512</v>
-      </c>
-      <c r="E59" s="5" t="s">
-        <v>1513</v>
       </c>
       <c r="F59" s="4" t="s">
         <v>1145</v>
@@ -83423,10 +83420,10 @@
         <v>37</v>
       </c>
       <c r="D60" s="4" t="s">
+        <v>1511</v>
+      </c>
+      <c r="E60" s="5" t="s">
         <v>1512</v>
-      </c>
-      <c r="E60" s="5" t="s">
-        <v>1513</v>
       </c>
       <c r="F60" s="4" t="s">
         <v>1145</v>
@@ -83465,10 +83462,10 @@
         <v>37</v>
       </c>
       <c r="D61" s="4" t="s">
+        <v>1513</v>
+      </c>
+      <c r="E61" s="5" t="s">
         <v>1514</v>
-      </c>
-      <c r="E61" s="5" t="s">
-        <v>1515</v>
       </c>
       <c r="F61" s="4" t="s">
         <v>1145</v>
@@ -83507,10 +83504,10 @@
         <v>37</v>
       </c>
       <c r="D62" s="4" t="s">
+        <v>1513</v>
+      </c>
+      <c r="E62" s="5" t="s">
         <v>1514</v>
-      </c>
-      <c r="E62" s="5" t="s">
-        <v>1515</v>
       </c>
       <c r="F62" s="4" t="s">
         <v>1145</v>
@@ -83549,10 +83546,10 @@
         <v>37</v>
       </c>
       <c r="D63" s="4" t="s">
+        <v>1515</v>
+      </c>
+      <c r="E63" s="5" t="s">
         <v>1516</v>
-      </c>
-      <c r="E63" s="5" t="s">
-        <v>1517</v>
       </c>
       <c r="F63" s="4" t="s">
         <v>1145</v>
@@ -83591,10 +83588,10 @@
         <v>37</v>
       </c>
       <c r="D64" s="4" t="s">
+        <v>1515</v>
+      </c>
+      <c r="E64" s="5" t="s">
         <v>1516</v>
-      </c>
-      <c r="E64" s="5" t="s">
-        <v>1517</v>
       </c>
       <c r="F64" s="4" t="s">
         <v>1145</v>
@@ -83633,10 +83630,10 @@
         <v>37</v>
       </c>
       <c r="D65" s="4" t="s">
+        <v>1517</v>
+      </c>
+      <c r="E65" s="5" t="s">
         <v>1518</v>
-      </c>
-      <c r="E65" s="5" t="s">
-        <v>1519</v>
       </c>
       <c r="F65" s="4" t="s">
         <v>1145</v>
@@ -83675,10 +83672,10 @@
         <v>37</v>
       </c>
       <c r="D66" s="4" t="s">
+        <v>1517</v>
+      </c>
+      <c r="E66" s="5" t="s">
         <v>1518</v>
-      </c>
-      <c r="E66" s="5" t="s">
-        <v>1519</v>
       </c>
       <c r="F66" s="4" t="s">
         <v>1145</v>
@@ -83717,10 +83714,10 @@
         <v>37</v>
       </c>
       <c r="D67" s="4" t="s">
+        <v>1519</v>
+      </c>
+      <c r="E67" s="5" t="s">
         <v>1520</v>
-      </c>
-      <c r="E67" s="5" t="s">
-        <v>1521</v>
       </c>
       <c r="F67" s="4" t="s">
         <v>1145</v>
@@ -83759,10 +83756,10 @@
         <v>37</v>
       </c>
       <c r="D68" s="4" t="s">
+        <v>1521</v>
+      </c>
+      <c r="E68" s="5" t="s">
         <v>1522</v>
-      </c>
-      <c r="E68" s="5" t="s">
-        <v>1523</v>
       </c>
       <c r="F68" s="4" t="s">
         <v>1145</v>
@@ -83801,10 +83798,10 @@
         <v>37</v>
       </c>
       <c r="D69" s="4" t="s">
+        <v>1523</v>
+      </c>
+      <c r="E69" s="5" t="s">
         <v>1524</v>
-      </c>
-      <c r="E69" s="5" t="s">
-        <v>1525</v>
       </c>
       <c r="F69" s="4" t="s">
         <v>1145</v>
@@ -83843,10 +83840,10 @@
         <v>37</v>
       </c>
       <c r="D70" s="4" t="s">
+        <v>1523</v>
+      </c>
+      <c r="E70" s="5" t="s">
         <v>1524</v>
-      </c>
-      <c r="E70" s="5" t="s">
-        <v>1525</v>
       </c>
       <c r="F70" s="4" t="s">
         <v>1145</v>
@@ -83885,10 +83882,10 @@
         <v>37</v>
       </c>
       <c r="D71" s="4" t="s">
+        <v>1525</v>
+      </c>
+      <c r="E71" s="5" t="s">
         <v>1526</v>
-      </c>
-      <c r="E71" s="5" t="s">
-        <v>1527</v>
       </c>
       <c r="F71" s="4" t="s">
         <v>1145</v>
@@ -83927,16 +83924,16 @@
         <v>37</v>
       </c>
       <c r="D72" s="4" t="s">
+        <v>1525</v>
+      </c>
+      <c r="E72" s="5" t="s">
         <v>1526</v>
-      </c>
-      <c r="E72" s="5" t="s">
-        <v>1527</v>
       </c>
       <c r="F72" s="4" t="s">
         <v>1145</v>
       </c>
       <c r="G72" s="4" t="s">
-        <v>1528</v>
+        <v>1527</v>
       </c>
       <c r="H72" s="4" t="s">
         <v>41</v>
@@ -83969,10 +83966,10 @@
         <v>37</v>
       </c>
       <c r="D73" s="4" t="s">
+        <v>1528</v>
+      </c>
+      <c r="E73" s="5" t="s">
         <v>1529</v>
-      </c>
-      <c r="E73" s="5" t="s">
-        <v>1530</v>
       </c>
       <c r="F73" s="4" t="s">
         <v>1145</v>
@@ -84011,10 +84008,10 @@
         <v>37</v>
       </c>
       <c r="D74" s="4" t="s">
+        <v>1528</v>
+      </c>
+      <c r="E74" s="5" t="s">
         <v>1529</v>
-      </c>
-      <c r="E74" s="5" t="s">
-        <v>1530</v>
       </c>
       <c r="F74" s="4" t="s">
         <v>1145</v>
@@ -84053,10 +84050,10 @@
         <v>37</v>
       </c>
       <c r="D75" s="4" t="s">
+        <v>1530</v>
+      </c>
+      <c r="E75" s="5" t="s">
         <v>1531</v>
-      </c>
-      <c r="E75" s="5" t="s">
-        <v>1532</v>
       </c>
       <c r="F75" s="4" t="s">
         <v>1145</v>
@@ -84095,10 +84092,10 @@
         <v>37</v>
       </c>
       <c r="D76" s="4" t="s">
+        <v>1530</v>
+      </c>
+      <c r="E76" s="5" t="s">
         <v>1531</v>
-      </c>
-      <c r="E76" s="5" t="s">
-        <v>1532</v>
       </c>
       <c r="F76" s="4" t="s">
         <v>1145</v>
@@ -84137,10 +84134,10 @@
         <v>37</v>
       </c>
       <c r="D77" s="4" t="s">
+        <v>1530</v>
+      </c>
+      <c r="E77" s="5" t="s">
         <v>1531</v>
-      </c>
-      <c r="E77" s="5" t="s">
-        <v>1532</v>
       </c>
       <c r="F77" s="4" t="s">
         <v>1145</v>
@@ -84179,10 +84176,10 @@
         <v>37</v>
       </c>
       <c r="D78" s="4" t="s">
+        <v>1532</v>
+      </c>
+      <c r="E78" s="5" t="s">
         <v>1533</v>
-      </c>
-      <c r="E78" s="5" t="s">
-        <v>1534</v>
       </c>
       <c r="F78" s="4" t="s">
         <v>1145</v>
@@ -84221,10 +84218,10 @@
         <v>37</v>
       </c>
       <c r="D79" s="4" t="s">
+        <v>1532</v>
+      </c>
+      <c r="E79" s="5" t="s">
         <v>1533</v>
-      </c>
-      <c r="E79" s="5" t="s">
-        <v>1534</v>
       </c>
       <c r="F79" s="4" t="s">
         <v>1145</v>
@@ -84263,10 +84260,10 @@
         <v>37</v>
       </c>
       <c r="D80" s="4" t="s">
+        <v>1534</v>
+      </c>
+      <c r="E80" s="5" t="s">
         <v>1535</v>
-      </c>
-      <c r="E80" s="5" t="s">
-        <v>1536</v>
       </c>
       <c r="F80" s="4" t="s">
         <v>1145</v>
@@ -84305,16 +84302,16 @@
         <v>37</v>
       </c>
       <c r="D81" s="4" t="s">
+        <v>1534</v>
+      </c>
+      <c r="E81" s="5" t="s">
         <v>1535</v>
-      </c>
-      <c r="E81" s="5" t="s">
-        <v>1536</v>
       </c>
       <c r="F81" s="4" t="s">
         <v>1145</v>
       </c>
       <c r="G81" s="4" t="s">
-        <v>1528</v>
+        <v>1527</v>
       </c>
       <c r="H81" s="4" t="s">
         <v>96</v>
@@ -84347,10 +84344,10 @@
         <v>37</v>
       </c>
       <c r="D82" s="4" t="s">
+        <v>1536</v>
+      </c>
+      <c r="E82" s="5" t="s">
         <v>1537</v>
-      </c>
-      <c r="E82" s="5" t="s">
-        <v>1538</v>
       </c>
       <c r="F82" s="4" t="s">
         <v>1145</v>
@@ -84389,10 +84386,10 @@
         <v>37</v>
       </c>
       <c r="D83" s="4" t="s">
+        <v>1536</v>
+      </c>
+      <c r="E83" s="5" t="s">
         <v>1537</v>
-      </c>
-      <c r="E83" s="5" t="s">
-        <v>1538</v>
       </c>
       <c r="F83" s="4" t="s">
         <v>1145</v>
@@ -84431,10 +84428,10 @@
         <v>37</v>
       </c>
       <c r="D84" s="4" t="s">
+        <v>1538</v>
+      </c>
+      <c r="E84" s="5" t="s">
         <v>1539</v>
-      </c>
-      <c r="E84" s="5" t="s">
-        <v>1540</v>
       </c>
       <c r="F84" s="4" t="s">
         <v>734</v>
@@ -84473,10 +84470,10 @@
         <v>37</v>
       </c>
       <c r="D85" s="4" t="s">
+        <v>1538</v>
+      </c>
+      <c r="E85" s="5" t="s">
         <v>1539</v>
-      </c>
-      <c r="E85" s="5" t="s">
-        <v>1540</v>
       </c>
       <c r="F85" s="4" t="s">
         <v>734</v>
@@ -84515,10 +84512,10 @@
         <v>593</v>
       </c>
       <c r="D86" s="4" t="s">
+        <v>1540</v>
+      </c>
+      <c r="E86" s="5" t="s">
         <v>1541</v>
-      </c>
-      <c r="E86" s="5" t="s">
-        <v>1542</v>
       </c>
       <c r="F86" s="4" t="s">
         <v>710</v>
@@ -84557,10 +84554,10 @@
         <v>593</v>
       </c>
       <c r="D87" s="4" t="s">
+        <v>1540</v>
+      </c>
+      <c r="E87" s="5" t="s">
         <v>1541</v>
-      </c>
-      <c r="E87" s="5" t="s">
-        <v>1542</v>
       </c>
       <c r="F87" s="4" t="s">
         <v>710</v>
@@ -84599,10 +84596,10 @@
         <v>593</v>
       </c>
       <c r="D88" s="4" t="s">
+        <v>1542</v>
+      </c>
+      <c r="E88" s="5" t="s">
         <v>1543</v>
-      </c>
-      <c r="E88" s="5" t="s">
-        <v>1544</v>
       </c>
       <c r="F88" s="4" t="s">
         <v>710</v>
@@ -84641,10 +84638,10 @@
         <v>593</v>
       </c>
       <c r="D89" s="4" t="s">
+        <v>1542</v>
+      </c>
+      <c r="E89" s="5" t="s">
         <v>1543</v>
-      </c>
-      <c r="E89" s="5" t="s">
-        <v>1544</v>
       </c>
       <c r="F89" s="4" t="s">
         <v>710</v>

</xml_diff>